<commit_message>
Updated production data for Fox Complex
</commit_message>
<xml_diff>
--- a/data/Mappings/mapping_npri.xlsx
+++ b/data/Mappings/mapping_npri.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://polymtlca-my.sharepoint.com/personal/marin_pellan_polymtl_ca/Documents/POST_DOC/CODE/metallican_db/data/Mappings/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="69" documentId="13_ncr:1_{79931472-8B2F-4982-8306-AF8D7544F4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{79F3E67D-279D-4663-B2A3-B2BF2D31F971}"/>
+  <xr:revisionPtr revIDLastSave="75" documentId="13_ncr:1_{79931472-8B2F-4982-8306-AF8D7544F4B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B2D7F925-9911-41D5-9D40-8FC9727F9A65}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-705" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-705" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="mapping" sheetId="1" r:id="rId1"/>
@@ -2398,11 +2398,10 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2687,11 +2686,12 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr filterMode="1"/>
   <dimension ref="A1:B108"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="9.26953125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.08984375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.08984375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2" x14ac:dyDescent="0.35">
@@ -2702,7 +2702,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>444</v>
       </c>
@@ -2710,7 +2710,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="3" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A3">
         <v>1070</v>
       </c>
@@ -2718,7 +2718,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="4" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A4">
         <v>1071</v>
       </c>
@@ -2726,7 +2726,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="5" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A5">
         <v>1106</v>
       </c>
@@ -2734,7 +2734,7 @@
         <v>91</v>
       </c>
     </row>
-    <row r="6" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A6">
         <v>1148</v>
       </c>
@@ -2742,7 +2742,7 @@
         <v>84</v>
       </c>
     </row>
-    <row r="7" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A7">
         <v>1149</v>
       </c>
@@ -2750,7 +2750,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="8" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A8">
         <v>1233</v>
       </c>
@@ -2758,7 +2758,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="9" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A9">
         <v>1236</v>
       </c>
@@ -2766,7 +2766,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="10" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A10">
         <v>1303</v>
       </c>
@@ -2774,7 +2774,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="11" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A11">
         <v>1465</v>
       </c>
@@ -2782,7 +2782,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="12" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A12" s="1">
         <v>1467</v>
       </c>
@@ -2790,7 +2790,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="13" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A13">
         <v>1471</v>
       </c>
@@ -2798,7 +2798,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="14" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A14">
         <v>1520</v>
       </c>
@@ -2806,7 +2806,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="15" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A15">
         <v>1568</v>
       </c>
@@ -2814,7 +2814,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="16" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A16">
         <v>1651</v>
       </c>
@@ -2822,7 +2822,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A17">
         <v>1941</v>
       </c>
@@ -2830,7 +2830,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A18">
         <v>2000</v>
       </c>
@@ -2838,7 +2838,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A19">
         <v>2038</v>
       </c>
@@ -2846,7 +2846,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A20">
         <v>2100</v>
       </c>
@@ -2854,7 +2854,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="21" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A21">
         <v>2132</v>
       </c>
@@ -2862,7 +2862,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A22">
         <v>2372</v>
       </c>
@@ -2870,7 +2870,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A23">
         <v>2710</v>
       </c>
@@ -2878,7 +2878,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A24">
         <v>2740</v>
       </c>
@@ -2886,7 +2886,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A25">
         <v>2978</v>
       </c>
@@ -2894,7 +2894,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A26">
         <v>2984</v>
       </c>
@@ -2902,7 +2902,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A27">
         <v>2986</v>
       </c>
@@ -2910,7 +2910,7 @@
         <v>38</v>
       </c>
     </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A28">
         <v>3060</v>
       </c>
@@ -2918,7 +2918,7 @@
         <v>13</v>
       </c>
     </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A29">
         <v>3062</v>
       </c>
@@ -2926,7 +2926,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A30">
         <v>3158</v>
       </c>
@@ -2934,7 +2934,7 @@
         <v>19</v>
       </c>
     </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A31">
         <v>3197</v>
       </c>
@@ -2942,7 +2942,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A32">
         <v>3356</v>
       </c>
@@ -2950,7 +2950,7 @@
         <v>83</v>
       </c>
     </row>
-    <row r="33" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A33">
         <v>3406</v>
       </c>
@@ -2958,7 +2958,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="34" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A34">
         <v>3411</v>
       </c>
@@ -2966,7 +2966,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="35" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A35">
         <v>3598</v>
       </c>
@@ -2974,7 +2974,7 @@
         <v>44</v>
       </c>
     </row>
-    <row r="36" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A36">
         <v>3623</v>
       </c>
@@ -2982,7 +2982,7 @@
         <v>67</v>
       </c>
     </row>
-    <row r="37" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A37">
         <v>3649</v>
       </c>
@@ -2990,7 +2990,7 @@
         <v>71</v>
       </c>
     </row>
-    <row r="38" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A38">
         <v>3713</v>
       </c>
@@ -2998,7 +2998,7 @@
         <v>74</v>
       </c>
     </row>
-    <row r="39" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A39">
         <v>3802</v>
       </c>
@@ -3014,7 +3014,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="41" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A41">
         <v>3824</v>
       </c>
@@ -3022,7 +3022,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="42" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A42">
         <v>3916</v>
       </c>
@@ -3030,7 +3030,7 @@
         <v>59</v>
       </c>
     </row>
-    <row r="43" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A43">
         <v>3991</v>
       </c>
@@ -3038,7 +3038,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="44" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A44">
         <v>4045</v>
       </c>
@@ -3046,7 +3046,7 @@
         <v>66</v>
       </c>
     </row>
-    <row r="45" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A45">
         <v>4169</v>
       </c>
@@ -3054,7 +3054,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="46" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A46">
         <v>4197</v>
       </c>
@@ -3062,7 +3062,7 @@
         <v>76</v>
       </c>
     </row>
-    <row r="47" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A47">
         <v>4778</v>
       </c>
@@ -3070,7 +3070,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="48" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A48">
         <v>4782</v>
       </c>
@@ -3078,7 +3078,7 @@
         <v>29</v>
       </c>
     </row>
-    <row r="49" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A49">
         <v>4806</v>
       </c>
@@ -3086,7 +3086,7 @@
         <v>61</v>
       </c>
     </row>
-    <row r="50" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A50">
         <v>4866</v>
       </c>
@@ -3094,7 +3094,7 @@
         <v>96</v>
       </c>
     </row>
-    <row r="51" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A51">
         <v>4868</v>
       </c>
@@ -3102,7 +3102,7 @@
         <v>3</v>
       </c>
     </row>
-    <row r="52" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A52">
         <v>5013</v>
       </c>
@@ -3110,7 +3110,7 @@
         <v>95</v>
       </c>
     </row>
-    <row r="53" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A53">
         <v>5102</v>
       </c>
@@ -3118,7 +3118,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="54" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A54">
         <v>5219</v>
       </c>
@@ -3126,7 +3126,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="55" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A55">
         <v>5448</v>
       </c>
@@ -3134,7 +3134,7 @@
         <v>62</v>
       </c>
     </row>
-    <row r="56" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A56">
         <v>5460</v>
       </c>
@@ -3142,7 +3142,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="57" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A57">
         <v>5510</v>
       </c>
@@ -3150,7 +3150,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="58" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A58">
         <v>5656</v>
       </c>
@@ -3158,7 +3158,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="59" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A59">
         <v>6093</v>
       </c>
@@ -3166,7 +3166,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="60" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A60">
         <v>6217</v>
       </c>
@@ -3174,7 +3174,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="61" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A61">
         <v>6344</v>
       </c>
@@ -3182,7 +3182,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="62" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A62">
         <v>8015</v>
       </c>
@@ -3190,7 +3190,7 @@
         <v>50</v>
       </c>
     </row>
-    <row r="63" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A63">
         <v>8757</v>
       </c>
@@ -3198,7 +3198,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="64" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A64">
         <v>8778</v>
       </c>
@@ -3206,7 +3206,7 @@
         <v>53</v>
       </c>
     </row>
-    <row r="65" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A65">
         <v>8783</v>
       </c>
@@ -3214,7 +3214,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="66" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A66">
         <v>8803</v>
       </c>
@@ -3222,7 +3222,7 @@
         <v>82</v>
       </c>
     </row>
-    <row r="67" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A67">
         <v>8807</v>
       </c>
@@ -3230,7 +3230,7 @@
         <v>15</v>
       </c>
     </row>
-    <row r="68" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A68">
         <v>10010</v>
       </c>
@@ -3238,7 +3238,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="69" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A69">
         <v>10153</v>
       </c>
@@ -3246,7 +3246,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="70" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A70">
         <v>10199</v>
       </c>
@@ -3254,7 +3254,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="71" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A71">
         <v>10201</v>
       </c>
@@ -3262,7 +3262,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="72" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A72">
         <v>10202</v>
       </c>
@@ -3270,7 +3270,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="73" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A73" s="1">
         <v>10203</v>
       </c>
@@ -3278,7 +3278,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="74" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A74" s="1">
         <v>10204</v>
       </c>
@@ -3286,7 +3286,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="75" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A75">
         <v>11123</v>
       </c>
@@ -3294,7 +3294,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="76" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A76">
         <v>11154</v>
       </c>
@@ -3302,7 +3302,7 @@
         <v>17</v>
       </c>
     </row>
-    <row r="77" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A77">
         <v>11454</v>
       </c>
@@ -3310,7 +3310,7 @@
         <v>85</v>
       </c>
     </row>
-    <row r="78" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A78">
         <v>11588</v>
       </c>
@@ -3318,7 +3318,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="79" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A79">
         <v>11794</v>
       </c>
@@ -3326,7 +3326,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="80" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A80">
         <v>11796</v>
       </c>
@@ -3334,7 +3334,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A81">
         <v>11867</v>
       </c>
@@ -3342,7 +3342,7 @@
         <v>68</v>
       </c>
     </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A82">
         <v>11878</v>
       </c>
@@ -3350,7 +3350,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A83">
         <v>19397</v>
       </c>
@@ -3358,7 +3358,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A84">
         <v>20131</v>
       </c>
@@ -3366,7 +3366,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A85">
         <v>23273</v>
       </c>
@@ -3374,7 +3374,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A86">
         <v>24216</v>
       </c>
@@ -3382,7 +3382,7 @@
         <v>70</v>
       </c>
     </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A87">
         <v>25188</v>
       </c>
@@ -3390,7 +3390,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A88">
         <v>25434</v>
       </c>
@@ -3398,7 +3398,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A89">
         <v>26132</v>
       </c>
@@ -3406,7 +3406,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A90">
         <v>26423</v>
       </c>
@@ -3414,7 +3414,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A91">
         <v>27063</v>
       </c>
@@ -3422,7 +3422,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A92">
         <v>27853</v>
       </c>
@@ -3430,7 +3430,7 @@
         <v>56</v>
       </c>
     </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A93">
         <v>28726</v>
       </c>
@@ -3438,7 +3438,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A94">
         <v>28761</v>
       </c>
@@ -3446,7 +3446,7 @@
         <v>33</v>
       </c>
     </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A95">
         <v>29072</v>
       </c>
@@ -3454,7 +3454,7 @@
         <v>86</v>
       </c>
     </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A96">
         <v>29191</v>
       </c>
@@ -3462,7 +3462,7 @@
         <v>79</v>
       </c>
     </row>
-    <row r="97" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A97">
         <v>29548</v>
       </c>
@@ -3470,7 +3470,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="98" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A98">
         <v>29877</v>
       </c>
@@ -3478,7 +3478,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="99" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A99">
         <v>30798</v>
       </c>
@@ -3486,7 +3486,7 @@
         <v>88</v>
       </c>
     </row>
-    <row r="100" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A100">
         <v>32235</v>
       </c>
@@ -3494,7 +3494,7 @@
         <v>90</v>
       </c>
     </row>
-    <row r="101" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A101">
         <v>32933</v>
       </c>
@@ -3502,7 +3502,7 @@
         <v>52</v>
       </c>
     </row>
-    <row r="102" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A102">
         <v>33049</v>
       </c>
@@ -3510,7 +3510,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="103" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A103">
         <v>33819</v>
       </c>
@@ -3518,7 +3518,7 @@
         <v>77</v>
       </c>
     </row>
-    <row r="104" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A104">
         <v>34014</v>
       </c>
@@ -3526,7 +3526,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="105" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A105" s="1">
         <v>99</v>
       </c>
@@ -3534,7 +3534,7 @@
         <v>120</v>
       </c>
     </row>
-    <row r="106" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A106" s="1">
         <v>29389</v>
       </c>
@@ -3542,7 +3542,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="107" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A107" s="1">
         <v>8600</v>
       </c>
@@ -3550,7 +3550,7 @@
         <v>389</v>
       </c>
     </row>
-    <row r="108" spans="1:2" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:2" hidden="1" x14ac:dyDescent="0.35">
       <c r="A108" s="1">
         <v>32238</v>
       </c>
@@ -3560,6 +3560,11 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:B108" xr:uid="{00000000-0001-0000-0000-000000000000}">
+    <filterColumn colId="1">
+      <filters>
+        <filter val="ON-MAIN-4e0734b5"/>
+      </filters>
+    </filterColumn>
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:B104">
       <sortCondition ref="A1:A104"/>
     </sortState>
@@ -3575,8 +3580,8 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.7265625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="18" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="8.81640625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.54296875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.26953125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.90625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="35.81640625" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="63.6328125" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.453125" bestFit="1" customWidth="1"/>
@@ -7419,16 +7424,16 @@
       <c r="C198">
         <v>5713.75</v>
       </c>
-      <c r="D198" s="3" t="s">
+      <c r="D198" t="s">
         <v>370</v>
       </c>
-      <c r="E198" s="3" t="s">
+      <c r="E198" t="s">
         <v>357</v>
       </c>
-      <c r="F198" s="3">
+      <c r="F198">
         <v>72</v>
       </c>
-      <c r="G198" s="3">
+      <c r="G198">
         <v>70</v>
       </c>
     </row>
@@ -9711,7 +9716,7 @@
         <v>499</v>
       </c>
     </row>
-    <row r="317" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="317" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A317" t="s">
         <v>500</v>
       </c>
@@ -9780,7 +9785,7 @@
         <v>32.258064516128997</v>
       </c>
     </row>
-    <row r="320" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="320" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A320" t="s">
         <v>505</v>
       </c>
@@ -9872,7 +9877,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="324" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="324" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A324" t="s">
         <v>49</v>
       </c>
@@ -10160,7 +10165,7 @@
         <v>542</v>
       </c>
     </row>
-    <row r="345" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="345" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
       <c r="A345" t="s">
         <v>97</v>
       </c>
@@ -10229,7 +10234,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="348" spans="1:7" hidden="1" x14ac:dyDescent="0.35">
+    <row r="348" spans="1:7" x14ac:dyDescent="0.35">
       <c r="A348" t="s">
         <v>60</v>
       </c>
@@ -14387,9 +14392,9 @@
     </row>
   </sheetData>
   <autoFilter ref="A1:G589" xr:uid="{556460DC-71F1-43FF-BD31-36D25365B781}">
-    <filterColumn colId="1">
+    <filterColumn colId="3">
       <filters>
-        <filter val="2815"/>
+        <filter val="Timmins West"/>
       </filters>
     </filterColumn>
   </autoFilter>

</xml_diff>